<commit_message>
Build q2388 remote tile shard resume DAG
</commit_message>
<xml_diff>
--- a/task/关键标准答案.xlsx
+++ b/task/关键标准答案.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R3338c13baabd4cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="R2f4518ec123e4767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R4c4d7c9e6f994aed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="Rcb873c7a539a42a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R6b421d34917441d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R2fe1d88a1ef84d4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="R86bdb1498d344116"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R5601d604e1d544b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="R63a918b197ef49c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="Rb0bbb5b26be24dea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -378,10 +378,10 @@
         <x:v>Checkpoint</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>output/checkpoints下按family和shard_id保存</x:v>
+        <x:v>output/checkpoints</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
-        <x:v>保留可复用分片状态</x:v>
+        <x:v>按family和shard_id保留可复用分片状态</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
         <x:v>与processing_contract.json和处理账比较</x:v>
@@ -491,7 +491,7 @@
         <x:v>映射任务</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>task_id</x:v>
+        <x:v>Airflow对象名称</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
         <x:v>process_shard</x:v>
@@ -505,7 +505,7 @@
         <x:v>汇总任务</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>task_id</x:v>
+        <x:v>Airflow对象名称</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
         <x:v>summarize_batch</x:v>

</xml_diff>